<commit_message>
Remove tender-level exchange rate from template
</commit_message>
<xml_diff>
--- a/Tender_Template_ItemExchangeRate.xlsx
+++ b/Tender_Template_ItemExchangeRate.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -427,121 +427,169 @@
         <v>TND-2024-001</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ኮድ</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C3" t="str">
+        <v>የተያዘበት ቀን</v>
+      </c>
+      <c r="D3" t="str">
+        <v>የተያዘበት ቦታ</v>
+      </c>
+      <c r="E3" t="str">
+        <v>ያዥው አካል</v>
+      </c>
+      <c r="F3" t="str">
+        <v>ሞዴል</v>
+      </c>
+      <c r="G3" t="str">
+        <v>የእቃው አይነት</v>
+      </c>
+      <c r="H3" t="str">
+        <v>ማርክ</v>
+      </c>
+      <c r="I3" t="str">
+        <v>ስሪት ሀገር</v>
+      </c>
+      <c r="J3" t="str">
+        <v>መለኪያ</v>
+      </c>
+      <c r="K3" t="str">
+        <v>መጋዘን 1</v>
+      </c>
+      <c r="L3" t="str">
+        <v>መጋዘን 2</v>
+      </c>
+      <c r="M3" t="str">
+        <v>መጋዘን 3</v>
+      </c>
+      <c r="N3" t="str">
+        <v>ጠቅላላ ድምር</v>
+      </c>
+      <c r="O3" t="str">
+        <v>(FOB)</v>
+      </c>
+      <c r="P3" t="str">
+        <v>(CIF)</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>(TAX)</v>
+      </c>
+      <c r="R3" t="str">
         <v>Exchange Rate</v>
-      </c>
-      <c r="B2" t="str">
-        <v>120.50</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ኮድ</v>
+        <v>ኮድ-10</v>
       </c>
       <c r="B4" t="str">
-        <v>Title</v>
+        <v>Electronics Group</v>
       </c>
       <c r="C4" t="str">
-        <v>የተያዘበት ቀን</v>
+        <v>15-01-2024</v>
       </c>
       <c r="D4" t="str">
-        <v>የተያዘበት ቦታ</v>
+        <v>Dire Dawa</v>
       </c>
       <c r="E4" t="str">
-        <v>ያዥው አካል</v>
+        <v>Customs Authority</v>
       </c>
       <c r="F4" t="str">
-        <v>ሞዴል</v>
+        <v>52155001</v>
       </c>
       <c r="G4" t="str">
-        <v>የእቃው አይነት</v>
+        <v>Laptop</v>
       </c>
       <c r="H4" t="str">
-        <v>ማርክ</v>
+        <v>Dell</v>
       </c>
       <c r="I4" t="str">
-        <v>ስሪት ሀገር</v>
+        <v>USA</v>
       </c>
       <c r="J4" t="str">
-        <v>መለኪያ</v>
-      </c>
-      <c r="K4" t="str">
-        <v>መጋዘን 1</v>
-      </c>
-      <c r="L4" t="str">
-        <v>መጋዘን 2</v>
-      </c>
-      <c r="M4" t="str">
-        <v>መጋዘን 3</v>
-      </c>
-      <c r="N4" t="str">
-        <v>ጠቅላላ ድምር</v>
-      </c>
-      <c r="O4" t="str">
-        <v>(FOB)</v>
-      </c>
-      <c r="P4" t="str">
-        <v>(CIF)</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>(TAX)</v>
-      </c>
-      <c r="R4" t="str">
-        <v>Exchange Rate</v>
+        <v>EA</v>
+      </c>
+      <c r="K4">
+        <v>5</v>
+      </c>
+      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4">
+        <v>10</v>
+      </c>
+      <c r="O4">
+        <v>800</v>
+      </c>
+      <c r="P4">
+        <v>850</v>
+      </c>
+      <c r="Q4">
+        <v>900</v>
+      </c>
+      <c r="R4">
+        <v>120.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ኮድ-10</v>
+        <v/>
       </c>
       <c r="B5" t="str">
-        <v>Electronics Group</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>15-01-2024</v>
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>Dire Dawa</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>Customs Authority</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>52155001</v>
+        <v>52155002</v>
       </c>
       <c r="G5" t="str">
-        <v>Laptop</v>
+        <v>Monitor</v>
       </c>
       <c r="H5" t="str">
-        <v>Dell</v>
+        <v>Samsung</v>
       </c>
       <c r="I5" t="str">
-        <v>USA</v>
+        <v>Korea</v>
       </c>
       <c r="J5" t="str">
         <v>EA</v>
       </c>
       <c r="K5">
+        <v>10</v>
+      </c>
+      <c r="L5">
         <v>5</v>
       </c>
-      <c r="L5">
-        <v>3</v>
-      </c>
       <c r="M5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N5">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="O5">
-        <v>800</v>
+        <v>200</v>
       </c>
       <c r="P5">
-        <v>850</v>
+        <v>220</v>
       </c>
       <c r="Q5">
-        <v>900</v>
+        <v>250</v>
       </c>
       <c r="R5">
         <v>120.5</v>
@@ -564,40 +612,40 @@
         <v/>
       </c>
       <c r="F6" t="str">
-        <v>52155002</v>
+        <v>52155003</v>
       </c>
       <c r="G6" t="str">
-        <v>Monitor</v>
+        <v>Keyboard</v>
       </c>
       <c r="H6" t="str">
-        <v>Samsung</v>
+        <v>Logitech</v>
       </c>
       <c r="I6" t="str">
-        <v>Korea</v>
+        <v>China</v>
       </c>
       <c r="J6" t="str">
         <v>EA</v>
       </c>
       <c r="K6">
+        <v>15</v>
+      </c>
+      <c r="L6">
         <v>10</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
       </c>
       <c r="M6">
         <v>5</v>
       </c>
       <c r="N6">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="O6">
-        <v>200</v>
+        <v>30</v>
       </c>
       <c r="P6">
-        <v>220</v>
+        <v>35</v>
       </c>
       <c r="Q6">
-        <v>250</v>
+        <v>40</v>
       </c>
       <c r="R6">
         <v>120.5</v>
@@ -620,10 +668,10 @@
         <v/>
       </c>
       <c r="F7" t="str">
-        <v>52155003</v>
+        <v>52155004</v>
       </c>
       <c r="G7" t="str">
-        <v>Keyboard</v>
+        <v>Mouse</v>
       </c>
       <c r="H7" t="str">
         <v>Logitech</v>
@@ -635,25 +683,25 @@
         <v>EA</v>
       </c>
       <c r="K7">
+        <v>20</v>
+      </c>
+      <c r="L7">
         <v>15</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>10</v>
       </c>
-      <c r="M7">
-        <v>5</v>
-      </c>
       <c r="N7">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="O7">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="P7">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="Q7">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="R7">
         <v>120.5</v>
@@ -676,40 +724,40 @@
         <v/>
       </c>
       <c r="F8" t="str">
-        <v>52155004</v>
+        <v>52155005</v>
       </c>
       <c r="G8" t="str">
-        <v>Mouse</v>
+        <v>Printer</v>
       </c>
       <c r="H8" t="str">
-        <v>Logitech</v>
+        <v>HP</v>
       </c>
       <c r="I8" t="str">
-        <v>China</v>
+        <v>USA</v>
       </c>
       <c r="J8" t="str">
         <v>EA</v>
       </c>
       <c r="K8">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="L8">
+        <v>4</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+      <c r="N8">
         <v>15</v>
       </c>
-      <c r="M8">
-        <v>10</v>
-      </c>
-      <c r="N8">
-        <v>45</v>
-      </c>
       <c r="O8">
-        <v>15</v>
+        <v>300</v>
       </c>
       <c r="P8">
-        <v>18</v>
+        <v>320</v>
       </c>
       <c r="Q8">
-        <v>22</v>
+        <v>350</v>
       </c>
       <c r="R8">
         <v>120.5</v>
@@ -732,40 +780,40 @@
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>52155005</v>
+        <v>52155006</v>
       </c>
       <c r="G9" t="str">
-        <v>Printer</v>
+        <v>Scanner</v>
       </c>
       <c r="H9" t="str">
-        <v>HP</v>
+        <v>Canon</v>
       </c>
       <c r="I9" t="str">
-        <v>USA</v>
+        <v>Japan</v>
       </c>
       <c r="J9" t="str">
         <v>EA</v>
       </c>
       <c r="K9">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L9">
         <v>4</v>
       </c>
       <c r="M9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="O9">
+        <v>250</v>
+      </c>
+      <c r="P9">
+        <v>270</v>
+      </c>
+      <c r="Q9">
         <v>300</v>
-      </c>
-      <c r="P9">
-        <v>320</v>
-      </c>
-      <c r="Q9">
-        <v>350</v>
       </c>
       <c r="R9">
         <v>120.5</v>
@@ -788,40 +836,40 @@
         <v/>
       </c>
       <c r="F10" t="str">
-        <v>52155006</v>
+        <v>52155007</v>
       </c>
       <c r="G10" t="str">
-        <v>Scanner</v>
+        <v>Webcam</v>
       </c>
       <c r="H10" t="str">
-        <v>Canon</v>
+        <v>Logitech</v>
       </c>
       <c r="I10" t="str">
-        <v>Japan</v>
+        <v>China</v>
       </c>
       <c r="J10" t="str">
         <v>EA</v>
       </c>
       <c r="K10">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="L10">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N10">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="O10">
-        <v>250</v>
+        <v>50</v>
       </c>
       <c r="P10">
-        <v>270</v>
+        <v>55</v>
       </c>
       <c r="Q10">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="R10">
         <v>120.5</v>
@@ -844,40 +892,40 @@
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>52155007</v>
+        <v>52155008</v>
       </c>
       <c r="G11" t="str">
-        <v>Webcam</v>
+        <v>Headset</v>
       </c>
       <c r="H11" t="str">
-        <v>Logitech</v>
+        <v>Sony</v>
       </c>
       <c r="I11" t="str">
-        <v>China</v>
+        <v>Japan</v>
       </c>
       <c r="J11" t="str">
         <v>EA</v>
       </c>
       <c r="K11">
+        <v>18</v>
+      </c>
+      <c r="L11">
         <v>12</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>8</v>
       </c>
-      <c r="M11">
-        <v>5</v>
-      </c>
       <c r="N11">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="O11">
+        <v>40</v>
+      </c>
+      <c r="P11">
+        <v>45</v>
+      </c>
+      <c r="Q11">
         <v>50</v>
-      </c>
-      <c r="P11">
-        <v>55</v>
-      </c>
-      <c r="Q11">
-        <v>60</v>
       </c>
       <c r="R11">
         <v>120.5</v>
@@ -900,40 +948,40 @@
         <v/>
       </c>
       <c r="F12" t="str">
-        <v>52155008</v>
+        <v>52155009</v>
       </c>
       <c r="G12" t="str">
-        <v>Headset</v>
+        <v>USB Hub</v>
       </c>
       <c r="H12" t="str">
-        <v>Sony</v>
+        <v>Belkin</v>
       </c>
       <c r="I12" t="str">
-        <v>Japan</v>
+        <v>USA</v>
       </c>
       <c r="J12" t="str">
         <v>EA</v>
       </c>
       <c r="K12">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="L12">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M12">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N12">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="O12">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="P12">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="Q12">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="R12">
         <v>120.5</v>
@@ -956,13 +1004,13 @@
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>52155009</v>
+        <v>52155010</v>
       </c>
       <c r="G13" t="str">
-        <v>USB Hub</v>
+        <v>External HDD</v>
       </c>
       <c r="H13" t="str">
-        <v>Belkin</v>
+        <v>Seagate</v>
       </c>
       <c r="I13" t="str">
         <v>USA</v>
@@ -971,137 +1019,137 @@
         <v>EA</v>
       </c>
       <c r="K13">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="L13">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="M13">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N13">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="O13">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="P13">
-        <v>22</v>
+        <v>85</v>
       </c>
       <c r="Q13">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="R13">
         <v>120.5</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
-      <c r="E14" t="str">
-        <v/>
-      </c>
-      <c r="F14" t="str">
-        <v>52155010</v>
-      </c>
-      <c r="G14" t="str">
-        <v>External HDD</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Seagate</v>
-      </c>
-      <c r="I14" t="str">
-        <v>USA</v>
-      </c>
-      <c r="J14" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K14">
+    <row r="15">
+      <c r="A15" t="str">
+        <v>ኮድ-20</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Office Supplies</v>
+      </c>
+      <c r="C15" t="str">
+        <v>16-01-2024</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Dire Dawa</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Customs Authority</v>
+      </c>
+      <c r="F15" t="str">
+        <v>52156001</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Paper A4</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Generic</v>
+      </c>
+      <c r="I15" t="str">
+        <v>India</v>
+      </c>
+      <c r="J15" t="str">
+        <v>BOX</v>
+      </c>
+      <c r="K15">
+        <v>50</v>
+      </c>
+      <c r="L15">
+        <v>30</v>
+      </c>
+      <c r="M15">
+        <v>20</v>
+      </c>
+      <c r="N15">
+        <v>100</v>
+      </c>
+      <c r="O15">
         <v>10</v>
       </c>
-      <c r="L14">
-        <v>8</v>
-      </c>
-      <c r="M14">
-        <v>6</v>
-      </c>
-      <c r="N14">
-        <v>24</v>
-      </c>
-      <c r="O14">
-        <v>80</v>
-      </c>
-      <c r="P14">
-        <v>85</v>
-      </c>
-      <c r="Q14">
-        <v>90</v>
-      </c>
-      <c r="R14">
-        <v>120.5</v>
+      <c r="P15">
+        <v>12</v>
+      </c>
+      <c r="Q15">
+        <v>15</v>
+      </c>
+      <c r="R15">
+        <v>121</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ኮድ-20</v>
+        <v/>
       </c>
       <c r="B16" t="str">
-        <v>Office Supplies</v>
+        <v/>
       </c>
       <c r="C16" t="str">
-        <v>16-01-2024</v>
+        <v/>
       </c>
       <c r="D16" t="str">
-        <v>Dire Dawa</v>
+        <v/>
       </c>
       <c r="E16" t="str">
-        <v>Customs Authority</v>
+        <v/>
       </c>
       <c r="F16" t="str">
-        <v>52156001</v>
+        <v>52156002</v>
       </c>
       <c r="G16" t="str">
-        <v>Paper A4</v>
+        <v>Pen</v>
       </c>
       <c r="H16" t="str">
-        <v>Generic</v>
+        <v>Pilot</v>
       </c>
       <c r="I16" t="str">
-        <v>India</v>
+        <v>Japan</v>
       </c>
       <c r="J16" t="str">
         <v>BOX</v>
       </c>
       <c r="K16">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="L16">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="M16">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N16">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="O16">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="P16">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="Q16">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="R16">
         <v>121</v>
@@ -1124,40 +1172,40 @@
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>52156002</v>
+        <v>52156003</v>
       </c>
       <c r="G17" t="str">
-        <v>Pen</v>
+        <v>Stapler</v>
       </c>
       <c r="H17" t="str">
-        <v>Pilot</v>
+        <v>Deli</v>
       </c>
       <c r="I17" t="str">
-        <v>Japan</v>
+        <v>China</v>
       </c>
       <c r="J17" t="str">
-        <v>BOX</v>
+        <v>EA</v>
       </c>
       <c r="K17">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L17">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="M17">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="N17">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="O17">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="P17">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="Q17">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="R17">
         <v>121</v>
@@ -1180,40 +1228,40 @@
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>52156003</v>
+        <v>52156004</v>
       </c>
       <c r="G18" t="str">
-        <v>Stapler</v>
+        <v>File Folder</v>
       </c>
       <c r="H18" t="str">
-        <v>Deli</v>
+        <v>Generic</v>
       </c>
       <c r="I18" t="str">
         <v>China</v>
       </c>
       <c r="J18" t="str">
-        <v>EA</v>
+        <v>BOX</v>
       </c>
       <c r="K18">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="L18">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="M18">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="N18">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="O18">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="P18">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q18">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="R18">
         <v>121</v>
@@ -1236,40 +1284,40 @@
         <v/>
       </c>
       <c r="F19" t="str">
-        <v>52156004</v>
+        <v>52156005</v>
       </c>
       <c r="G19" t="str">
-        <v>File Folder</v>
+        <v>Notebook</v>
       </c>
       <c r="H19" t="str">
         <v>Generic</v>
       </c>
       <c r="I19" t="str">
-        <v>China</v>
+        <v>India</v>
       </c>
       <c r="J19" t="str">
-        <v>BOX</v>
+        <v>EA</v>
       </c>
       <c r="K19">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="L19">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="M19">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="N19">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="O19">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="P19">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="Q19">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="R19">
         <v>121</v>
@@ -1292,40 +1340,40 @@
         <v/>
       </c>
       <c r="F20" t="str">
-        <v>52156005</v>
+        <v>52156006</v>
       </c>
       <c r="G20" t="str">
-        <v>Notebook</v>
+        <v>Marker</v>
       </c>
       <c r="H20" t="str">
-        <v>Generic</v>
+        <v>Sharpie</v>
       </c>
       <c r="I20" t="str">
-        <v>India</v>
+        <v>USA</v>
       </c>
       <c r="J20" t="str">
-        <v>EA</v>
+        <v>BOX</v>
       </c>
       <c r="K20">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="L20">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="M20">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="N20">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="O20">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="P20">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="Q20">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="R20">
         <v>121</v>
@@ -1348,40 +1396,40 @@
         <v/>
       </c>
       <c r="F21" t="str">
-        <v>52156006</v>
+        <v>52156007</v>
       </c>
       <c r="G21" t="str">
-        <v>Marker</v>
+        <v>Tape</v>
       </c>
       <c r="H21" t="str">
-        <v>Sharpie</v>
+        <v>3M</v>
       </c>
       <c r="I21" t="str">
         <v>USA</v>
       </c>
       <c r="J21" t="str">
-        <v>BOX</v>
+        <v>EA</v>
       </c>
       <c r="K21">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="L21">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="M21">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="N21">
-        <v>50</v>
+        <v>95</v>
       </c>
       <c r="O21">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="P21">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="Q21">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="R21">
         <v>121</v>
@@ -1404,40 +1452,40 @@
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>52156007</v>
+        <v>52156008</v>
       </c>
       <c r="G22" t="str">
-        <v>Tape</v>
+        <v>Scissors</v>
       </c>
       <c r="H22" t="str">
-        <v>3M</v>
+        <v>Generic</v>
       </c>
       <c r="I22" t="str">
-        <v>USA</v>
+        <v>China</v>
       </c>
       <c r="J22" t="str">
         <v>EA</v>
       </c>
       <c r="K22">
+        <v>20</v>
+      </c>
+      <c r="L22">
+        <v>15</v>
+      </c>
+      <c r="M22">
+        <v>10</v>
+      </c>
+      <c r="N22">
         <v>45</v>
       </c>
-      <c r="L22">
-        <v>30</v>
-      </c>
-      <c r="M22">
-        <v>20</v>
-      </c>
-      <c r="N22">
-        <v>95</v>
-      </c>
       <c r="O22">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="P22">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="Q22">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="R22">
         <v>121</v>
@@ -1460,40 +1508,40 @@
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>52156008</v>
+        <v>52156009</v>
       </c>
       <c r="G23" t="str">
-        <v>Scissors</v>
+        <v>Calculator</v>
       </c>
       <c r="H23" t="str">
-        <v>Generic</v>
+        <v>Casio</v>
       </c>
       <c r="I23" t="str">
-        <v>China</v>
+        <v>Japan</v>
       </c>
       <c r="J23" t="str">
         <v>EA</v>
       </c>
       <c r="K23">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="L23">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M23">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N23">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="O23">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="P23">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="Q23">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="R23">
         <v>121</v>
@@ -1516,152 +1564,152 @@
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>52156009</v>
+        <v>52156010</v>
       </c>
       <c r="G24" t="str">
-        <v>Calculator</v>
+        <v>Whiteboard</v>
       </c>
       <c r="H24" t="str">
-        <v>Casio</v>
+        <v>Generic</v>
       </c>
       <c r="I24" t="str">
-        <v>Japan</v>
+        <v>China</v>
       </c>
       <c r="J24" t="str">
         <v>EA</v>
       </c>
       <c r="K24">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="L24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M24">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N24">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="O24">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="P24">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="Q24">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="R24">
         <v>121</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v/>
-      </c>
-      <c r="B25" t="str">
-        <v/>
-      </c>
-      <c r="C25" t="str">
-        <v/>
-      </c>
-      <c r="D25" t="str">
-        <v/>
-      </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25" t="str">
-        <v>52156010</v>
-      </c>
-      <c r="G25" t="str">
-        <v>Whiteboard</v>
-      </c>
-      <c r="H25" t="str">
-        <v>Generic</v>
-      </c>
-      <c r="I25" t="str">
-        <v>China</v>
-      </c>
-      <c r="J25" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K25">
-        <v>10</v>
-      </c>
-      <c r="L25">
+    <row r="26">
+      <c r="A26" t="str">
+        <v>ኮድ-30</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Office Furniture</v>
+      </c>
+      <c r="C26" t="str">
+        <v>17-01-2024</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Dire Dawa</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Customs Authority</v>
+      </c>
+      <c r="F26" t="str">
+        <v>52157001</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Office Chair</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Herman Miller</v>
+      </c>
+      <c r="I26" t="str">
+        <v>USA</v>
+      </c>
+      <c r="J26" t="str">
+        <v>EA</v>
+      </c>
+      <c r="K26">
+        <v>12</v>
+      </c>
+      <c r="L26">
         <v>8</v>
       </c>
-      <c r="M25">
+      <c r="M26">
         <v>5</v>
       </c>
-      <c r="N25">
-        <v>23</v>
-      </c>
-      <c r="O25">
-        <v>40</v>
-      </c>
-      <c r="P25">
-        <v>45</v>
-      </c>
-      <c r="Q25">
-        <v>50</v>
-      </c>
-      <c r="R25">
-        <v>121</v>
+      <c r="N26">
+        <v>25</v>
+      </c>
+      <c r="O26">
+        <v>200</v>
+      </c>
+      <c r="P26">
+        <v>220</v>
+      </c>
+      <c r="Q26">
+        <v>250</v>
+      </c>
+      <c r="R26">
+        <v>119.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ኮድ-30</v>
+        <v/>
       </c>
       <c r="B27" t="str">
-        <v>Office Furniture</v>
+        <v/>
       </c>
       <c r="C27" t="str">
-        <v>17-01-2024</v>
+        <v/>
       </c>
       <c r="D27" t="str">
-        <v>Dire Dawa</v>
+        <v/>
       </c>
       <c r="E27" t="str">
-        <v>Customs Authority</v>
+        <v/>
       </c>
       <c r="F27" t="str">
-        <v>52157001</v>
+        <v>52157002</v>
       </c>
       <c r="G27" t="str">
-        <v>Office Chair</v>
+        <v>Desk</v>
       </c>
       <c r="H27" t="str">
-        <v>Herman Miller</v>
+        <v>IKEA</v>
       </c>
       <c r="I27" t="str">
-        <v>USA</v>
+        <v>Sweden</v>
       </c>
       <c r="J27" t="str">
         <v>EA</v>
       </c>
       <c r="K27">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L27">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N27">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="O27">
+        <v>150</v>
+      </c>
+      <c r="P27">
+        <v>170</v>
+      </c>
+      <c r="Q27">
         <v>200</v>
-      </c>
-      <c r="P27">
-        <v>220</v>
-      </c>
-      <c r="Q27">
-        <v>250</v>
       </c>
       <c r="R27">
         <v>119.5</v>
@@ -1684,40 +1732,40 @@
         <v/>
       </c>
       <c r="F28" t="str">
-        <v>52157002</v>
+        <v>52157003</v>
       </c>
       <c r="G28" t="str">
-        <v>Desk</v>
+        <v>Filing Cabinet</v>
       </c>
       <c r="H28" t="str">
-        <v>IKEA</v>
+        <v>Generic</v>
       </c>
       <c r="I28" t="str">
-        <v>Sweden</v>
+        <v>China</v>
       </c>
       <c r="J28" t="str">
         <v>EA</v>
       </c>
       <c r="K28">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M28">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N28">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="O28">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="P28">
-        <v>170</v>
+        <v>110</v>
       </c>
       <c r="Q28">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="R28">
         <v>119.5</v>
@@ -1740,40 +1788,40 @@
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>52157003</v>
+        <v>52157004</v>
       </c>
       <c r="G29" t="str">
-        <v>Filing Cabinet</v>
+        <v>Bookshelf</v>
       </c>
       <c r="H29" t="str">
-        <v>Generic</v>
+        <v>IKEA</v>
       </c>
       <c r="I29" t="str">
-        <v>China</v>
+        <v>Sweden</v>
       </c>
       <c r="J29" t="str">
         <v>EA</v>
       </c>
       <c r="K29">
+        <v>15</v>
+      </c>
+      <c r="L29">
+        <v>10</v>
+      </c>
+      <c r="M29">
         <v>8</v>
       </c>
-      <c r="L29">
-        <v>5</v>
-      </c>
-      <c r="M29">
-        <v>3</v>
-      </c>
       <c r="N29">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="O29">
+        <v>80</v>
+      </c>
+      <c r="P29">
+        <v>90</v>
+      </c>
+      <c r="Q29">
         <v>100</v>
-      </c>
-      <c r="P29">
-        <v>110</v>
-      </c>
-      <c r="Q29">
-        <v>130</v>
       </c>
       <c r="R29">
         <v>119.5</v>
@@ -1796,40 +1844,40 @@
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>52157004</v>
+        <v>52157005</v>
       </c>
       <c r="G30" t="str">
-        <v>Bookshelf</v>
+        <v>Conference Table</v>
       </c>
       <c r="H30" t="str">
-        <v>IKEA</v>
+        <v>Generic</v>
       </c>
       <c r="I30" t="str">
-        <v>Sweden</v>
+        <v>China</v>
       </c>
       <c r="J30" t="str">
         <v>EA</v>
       </c>
       <c r="K30">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L30">
+        <v>3</v>
+      </c>
+      <c r="M30">
+        <v>2</v>
+      </c>
+      <c r="N30">
         <v>10</v>
       </c>
-      <c r="M30">
-        <v>8</v>
-      </c>
-      <c r="N30">
-        <v>33</v>
-      </c>
       <c r="O30">
-        <v>80</v>
+        <v>300</v>
       </c>
       <c r="P30">
-        <v>90</v>
+        <v>330</v>
       </c>
       <c r="Q30">
-        <v>100</v>
+        <v>370</v>
       </c>
       <c r="R30">
         <v>119.5</v>
@@ -1852,10 +1900,10 @@
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>52157005</v>
+        <v>52157006</v>
       </c>
       <c r="G31" t="str">
-        <v>Conference Table</v>
+        <v>Meeting Chair</v>
       </c>
       <c r="H31" t="str">
         <v>Generic</v>
@@ -1867,25 +1915,25 @@
         <v>EA</v>
       </c>
       <c r="K31">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="L31">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="M31">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="N31">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="O31">
-        <v>300</v>
+        <v>50</v>
       </c>
       <c r="P31">
-        <v>330</v>
+        <v>55</v>
       </c>
       <c r="Q31">
-        <v>370</v>
+        <v>65</v>
       </c>
       <c r="R31">
         <v>119.5</v>
@@ -1908,13 +1956,13 @@
         <v/>
       </c>
       <c r="F32" t="str">
-        <v>52157006</v>
+        <v>52157007</v>
       </c>
       <c r="G32" t="str">
-        <v>Meeting Chair</v>
+        <v>Standing Desk</v>
       </c>
       <c r="H32" t="str">
-        <v>Generic</v>
+        <v>Flexispot</v>
       </c>
       <c r="I32" t="str">
         <v>China</v>
@@ -1923,25 +1971,25 @@
         <v>EA</v>
       </c>
       <c r="K32">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="L32">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="M32">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="N32">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="O32">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="P32">
-        <v>55</v>
+        <v>280</v>
       </c>
       <c r="Q32">
-        <v>65</v>
+        <v>320</v>
       </c>
       <c r="R32">
         <v>119.5</v>
@@ -1964,40 +2012,40 @@
         <v/>
       </c>
       <c r="F33" t="str">
-        <v>52157007</v>
+        <v>52157008</v>
       </c>
       <c r="G33" t="str">
-        <v>Standing Desk</v>
+        <v>Drawer Unit</v>
       </c>
       <c r="H33" t="str">
-        <v>Flexispot</v>
+        <v>IKEA</v>
       </c>
       <c r="I33" t="str">
-        <v>China</v>
+        <v>Sweden</v>
       </c>
       <c r="J33" t="str">
         <v>EA</v>
       </c>
       <c r="K33">
+        <v>12</v>
+      </c>
+      <c r="L33">
         <v>8</v>
       </c>
-      <c r="L33">
-        <v>5</v>
-      </c>
       <c r="M33">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N33">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="O33">
-        <v>250</v>
+        <v>60</v>
       </c>
       <c r="P33">
-        <v>280</v>
+        <v>70</v>
       </c>
       <c r="Q33">
-        <v>320</v>
+        <v>80</v>
       </c>
       <c r="R33">
         <v>119.5</v>
@@ -2020,40 +2068,40 @@
         <v/>
       </c>
       <c r="F34" t="str">
-        <v>52157008</v>
+        <v>52157009</v>
       </c>
       <c r="G34" t="str">
-        <v>Drawer Unit</v>
+        <v>Coat Rack</v>
       </c>
       <c r="H34" t="str">
-        <v>IKEA</v>
+        <v>Generic</v>
       </c>
       <c r="I34" t="str">
-        <v>Sweden</v>
+        <v>China</v>
       </c>
       <c r="J34" t="str">
         <v>EA</v>
       </c>
       <c r="K34">
+        <v>18</v>
+      </c>
+      <c r="L34">
         <v>12</v>
       </c>
-      <c r="L34">
+      <c r="M34">
         <v>8</v>
       </c>
-      <c r="M34">
-        <v>6</v>
-      </c>
       <c r="N34">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="O34">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="P34">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="Q34">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="R34">
         <v>119.5</v>
@@ -2076,10 +2124,10 @@
         <v/>
       </c>
       <c r="F35" t="str">
-        <v>52157009</v>
+        <v>52157010</v>
       </c>
       <c r="G35" t="str">
-        <v>Coat Rack</v>
+        <v>Waste Bin</v>
       </c>
       <c r="H35" t="str">
         <v>Generic</v>
@@ -2091,89 +2139,33 @@
         <v>EA</v>
       </c>
       <c r="K35">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="L35">
+        <v>30</v>
+      </c>
+      <c r="M35">
+        <v>20</v>
+      </c>
+      <c r="N35">
+        <v>90</v>
+      </c>
+      <c r="O35">
+        <v>10</v>
+      </c>
+      <c r="P35">
         <v>12</v>
       </c>
-      <c r="M35">
-        <v>8</v>
-      </c>
-      <c r="N35">
-        <v>38</v>
-      </c>
-      <c r="O35">
-        <v>30</v>
-      </c>
-      <c r="P35">
-        <v>35</v>
-      </c>
       <c r="Q35">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="R35">
         <v>119.5</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v/>
-      </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v/>
-      </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
-      <c r="E36" t="str">
-        <v/>
-      </c>
-      <c r="F36" t="str">
-        <v>52157010</v>
-      </c>
-      <c r="G36" t="str">
-        <v>Waste Bin</v>
-      </c>
-      <c r="H36" t="str">
-        <v>Generic</v>
-      </c>
-      <c r="I36" t="str">
-        <v>China</v>
-      </c>
-      <c r="J36" t="str">
-        <v>EA</v>
-      </c>
-      <c r="K36">
-        <v>40</v>
-      </c>
-      <c r="L36">
-        <v>30</v>
-      </c>
-      <c r="M36">
-        <v>20</v>
-      </c>
-      <c r="N36">
-        <v>90</v>
-      </c>
-      <c r="O36">
-        <v>10</v>
-      </c>
-      <c r="P36">
-        <v>12</v>
-      </c>
-      <c r="Q36">
-        <v>15</v>
-      </c>
-      <c r="R36">
-        <v>119.5</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add expireDate column to items
</commit_message>
<xml_diff>
--- a/Tender_Template_ItemExchangeRate.xlsx
+++ b/Tender_Template_ItemExchangeRate.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:S35"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -417,6 +417,7 @@
     <col min="16" max="16" width="10.83203125" customWidth="1"/>
     <col min="17" max="17" width="10.83203125" customWidth="1"/>
     <col min="18" max="18" width="15.83203125" customWidth="1"/>
+    <col min="19" max="19" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,6 +483,9 @@
       <c r="R3" t="str">
         <v>Exchange Rate</v>
       </c>
+      <c r="S3" t="str">
+        <v>የማብቂያ ቀን</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -538,6 +542,9 @@
       <c r="R4">
         <v>120.5</v>
       </c>
+      <c r="S4" t="str">
+        <v>31-12-2025</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -594,6 +601,9 @@
       <c r="R5">
         <v>120.5</v>
       </c>
+      <c r="S5" t="str">
+        <v>31-12-2025</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -650,6 +660,9 @@
       <c r="R6">
         <v>120.5</v>
       </c>
+      <c r="S6" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -706,6 +719,9 @@
       <c r="R7">
         <v>120.5</v>
       </c>
+      <c r="S7" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -762,6 +778,9 @@
       <c r="R8">
         <v>120.5</v>
       </c>
+      <c r="S8" t="str">
+        <v>31-12-2025</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -818,6 +837,9 @@
       <c r="R9">
         <v>120.5</v>
       </c>
+      <c r="S9" t="str">
+        <v>31-12-2025</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -874,6 +896,9 @@
       <c r="R10">
         <v>120.5</v>
       </c>
+      <c r="S10" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -930,6 +955,9 @@
       <c r="R11">
         <v>120.5</v>
       </c>
+      <c r="S11" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -986,6 +1014,9 @@
       <c r="R12">
         <v>120.5</v>
       </c>
+      <c r="S12" t="str">
+        <v>31-12-2025</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1041,6 +1072,9 @@
       </c>
       <c r="R13">
         <v>120.5</v>
+      </c>
+      <c r="S13" t="str">
+        <v>31-12-2025</v>
       </c>
     </row>
     <row r="15">
@@ -1098,6 +1132,9 @@
       <c r="R15">
         <v>121</v>
       </c>
+      <c r="S15" t="str">
+        <v>31-12-2027</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1154,6 +1191,9 @@
       <c r="R16">
         <v>121</v>
       </c>
+      <c r="S16" t="str">
+        <v>31-12-2027</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1210,6 +1250,9 @@
       <c r="R17">
         <v>121</v>
       </c>
+      <c r="S17" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1266,6 +1309,9 @@
       <c r="R18">
         <v>121</v>
       </c>
+      <c r="S18" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1322,6 +1368,9 @@
       <c r="R19">
         <v>121</v>
       </c>
+      <c r="S19" t="str">
+        <v>31-12-2027</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1378,6 +1427,9 @@
       <c r="R20">
         <v>121</v>
       </c>
+      <c r="S20" t="str">
+        <v>31-12-2027</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1434,6 +1486,9 @@
       <c r="R21">
         <v>121</v>
       </c>
+      <c r="S21" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1490,6 +1545,9 @@
       <c r="R22">
         <v>121</v>
       </c>
+      <c r="S22" t="str">
+        <v>31-12-2026</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1546,6 +1604,9 @@
       <c r="R23">
         <v>121</v>
       </c>
+      <c r="S23" t="str">
+        <v>31-12-2025</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1601,6 +1662,9 @@
       </c>
       <c r="R24">
         <v>121</v>
+      </c>
+      <c r="S24" t="str">
+        <v>31-12-2025</v>
       </c>
     </row>
     <row r="26">
@@ -1658,6 +1722,9 @@
       <c r="R26">
         <v>119.5</v>
       </c>
+      <c r="S26" t="str">
+        <v>31-12-2030</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1714,6 +1781,9 @@
       <c r="R27">
         <v>119.5</v>
       </c>
+      <c r="S27" t="str">
+        <v>31-12-2030</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1770,6 +1840,9 @@
       <c r="R28">
         <v>119.5</v>
       </c>
+      <c r="S28" t="str">
+        <v>31-12-2029</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1826,6 +1899,9 @@
       <c r="R29">
         <v>119.5</v>
       </c>
+      <c r="S29" t="str">
+        <v>31-12-2029</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1882,6 +1958,9 @@
       <c r="R30">
         <v>119.5</v>
       </c>
+      <c r="S30" t="str">
+        <v>31-12-2030</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1938,6 +2017,9 @@
       <c r="R31">
         <v>119.5</v>
       </c>
+      <c r="S31" t="str">
+        <v>31-12-2030</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1994,6 +2076,9 @@
       <c r="R32">
         <v>119.5</v>
       </c>
+      <c r="S32" t="str">
+        <v>31-12-2029</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2050,6 +2135,9 @@
       <c r="R33">
         <v>119.5</v>
       </c>
+      <c r="S33" t="str">
+        <v>31-12-2029</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2106,6 +2194,9 @@
       <c r="R34">
         <v>119.5</v>
       </c>
+      <c r="S34" t="str">
+        <v>31-12-2028</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2162,10 +2253,13 @@
       <c r="R35">
         <v>119.5</v>
       </c>
+      <c r="S35" t="str">
+        <v>31-12-2028</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>